<commit_message>
pmp rename edildi, kontrol listesi eklendi
</commit_message>
<xml_diff>
--- a/Docs/Proje Kontrol Listesi.xlsx
+++ b/Docs/Proje Kontrol Listesi.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="155">
   <si>
     <t>Proje Grubu adi:</t>
   </si>
@@ -339,9 +339,11 @@
   </si>
   <si>
     <t>IEEE_SRS v2.0
-Sayfa 4, Functional Requirements başlığı
-IEEE_STP v1.0.docx
-BURAYA DAHA SONRA BAKILACAK</t>
+Sayfa 4, Product Functions başlığı
+Sayfa 7-8, Software System Attributes başlığı</t>
+  </si>
+  <si>
+    <t>SRS dokümanındaki Product Functions başlığında ürünün sistem bağlamını. Temel gereksinimler belirtilmiştir. Software System Attributes başlığında ise temel metrikler yer alarak performans kritlerleri bulunmaktadır.</t>
   </si>
   <si>
     <t>2.3 User Characteristics</t>
@@ -396,6 +398,13 @@
     <t>Kullanıcı arayüzü gereksinimleri liste halinde açıkça tanımlanmış mı? Draft cizimler var mi</t>
   </si>
   <si>
+    <t>IEEE_SDD v1.1.docx
+Sayfa 3-19, System Overview ve Detailed Design başlıkları</t>
+  </si>
+  <si>
+    <t>SDD'deki bu bölümler kullanıcı arayüzünün işlevsel beklentilerini (dashboard, navigation tabs, real time updates) ve teknik altyapıyı (WebSocket, REST endpoints) açıklar. Aynı zamanda SDD içerisinde bulunan Class, Algorithm Flow, Sequence diagramlar ile de sistem akışı görselleştirilmiştir.</t>
+  </si>
+  <si>
     <t>ISO 9241-210</t>
   </si>
   <si>
@@ -405,24 +414,52 @@
     <t>Donanım arayüzleri ve uyumluluk gereksinimleri belirtilmiş mi? Donanim arayuzleri liste halinde girdi ve ciktilar detaylandirilarak verilmis mi? Ilgili standartlar ve ureticiler belirtilmis mi?</t>
   </si>
   <si>
+    <t>IEEE_SRS v2.0
+Sayfa 5, Constraints başlığı
+IEEE_SDD v1.1.docx
+Sayfa 22, Deployment Architecture başlığı</t>
+  </si>
+  <si>
+    <t>SRS içerisindeki Constraints başlığı altında hardware gereksinimlerinden bahsedilmiş olunup ve SDD'de dokümanında deployment diagram ile deployment şeması ve kullanılacak componentler belirtilmiştir. Dokümanlar donanım gereksinimlerini ve prototip dağıtımını tanımlar. Ancak donanım arayüzleri proje kapsamında kullanımı olmayacağından dolayı belgelendirilmemiştir.</t>
+  </si>
+  <si>
     <t>3.1.3 Software Interfaces</t>
   </si>
   <si>
     <t>Yazılım arayüzleri (API'ler, hizmetler vb.) dokümante edilmiş mi? Yazilim arayuzleri liste halinde girdi ve ciktilar detaylandirilarak verilmis mi? Ilgili standartlar ve ureticiler belirtilmis mi?</t>
   </si>
   <si>
+    <t>IEEE_SDD v1.1.docx
+Sayfa 9-14, Interface Descriptions ve Data Design başlıkları</t>
+  </si>
+  <si>
+    <t>SDD içerisindeki Interface Descriptions ve Data Design kısımlarında yazılım arayüzlerinin hangi bileşenler arasında olduğunu ve yüksek seviyedeki etkileşimleri açıklar. Beraberinde içerdiği class diagram ile görselleştirilmiştir.</t>
+  </si>
+  <si>
     <t>3.1.4 Communication Interfaces</t>
   </si>
   <si>
     <t>İletişim protokolleri ve veri formatları açıkça belirtilmiş mi? Protokol tanimi, state diagram, standart</t>
   </si>
   <si>
+    <t>IEEE_SAD v1.0
+Sayfa 4-7, Architectural Views başlığı
+IEEE_SDD v1.1.docx
+Sayfa 9-11, Interface Descriptions</t>
+  </si>
+  <si>
+    <t>SDD ve SAD dokümanlarında REST, WebSocket, MQ ve e‑posta/OAuth bağlantıları ve akış diyagramları detaylıca tanımlanmıştır.</t>
+  </si>
+  <si>
     <t>3.2 Functional Requirements</t>
   </si>
   <si>
     <t>Fonksiyonel gereksinimler kullanıcı senaryolarıyla uyumlu mu? Gereksinim numarasi kullanim durumu numarasi eslestirme matrisi</t>
   </si>
   <si>
+    <t>Yan hücrede eşleştirimiş matrix yer almaktadır:</t>
+  </si>
+  <si>
     <t>ISO/IEC/IEEE 29148</t>
   </si>
   <si>
@@ -432,18 +469,43 @@
     <t>Sistem performans kriterleri (tepki süresi, kapasite vb.) belirtilmiş mi?</t>
   </si>
   <si>
+    <t>IEEE_SRS v2.0
+Sayfa 7-8, Software System Attributes başlığı</t>
+  </si>
+  <si>
+    <t>SRS dokümanında yer alan Software System Attributes başlığının altında bulunan tabloda performans kriterleri mevcuttur. Temel metrikler yer almaktadır(IDS p95 ≤ 2s, dashboard ≤ 3s, malware inference p95 ≤ 5s, CVE fetch ≤ 12h, uptime ≥ 99%).</t>
+  </si>
+  <si>
     <t>3.4 Design Constraints</t>
   </si>
   <si>
     <t>Tasarım kısıtları (standartlar, donanım, yazılım vb.) açıkça tanımlanmış mı?</t>
   </si>
   <si>
+    <t>IEEE_SDD v1.1.docx
+Sayfa 3-5, System Overview başlığı
+IEEE_SRS v2.0
+Sayfa 6-8, Specific Requirements başlığı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDD ve SRS dokümanlarında temel tasarım kısıtları (monolitik mimari tercihi, kullanılan framework ve DB, prototip dağıtım kısıtları, bazı standart referansları) tanımlanmıştır. </t>
+  </si>
+  <si>
     <t>3.5.1 Reliability</t>
   </si>
   <si>
     <t>Sistemin güvenilirlik gereksinimleri tanımlanmış mı? Hata toleransi, hata frekansi, kurtarilabilirlik, sureklili tutarlilik, beklenmeyen durumlara karsi dayaniklilik, zamaninda tepki</t>
   </si>
   <si>
+    <t>IEEE_SRS v2.0
+Sayfa 7-8, Software System Attributes başlığı
+IEEE_STP v1.0.docx
+Sayfa 5, Pass/Fail Criteria</t>
+  </si>
+  <si>
+    <t>SRS'teki Software System Attributes başlığı altında bulunan tabloda bazı güvenilirlik hedefleri, kalite tanımları (ör. MTBF ≥ 100 saat, uptime ≥ 99%, veri hata oranı ≤ %0.5, iş akışı retry/queue yapısı, performans p95 hedefleri) mevcut. Aynı şekilde STP dosyasında bulunan Pass/Fail Criteria başlığında da testlerin nasıl bir sonuç karşısında pass veya fail durumlarının görüleceği tanımlanmıştır.</t>
+  </si>
+  <si>
     <t>ISO/IEC 25010</t>
   </si>
   <si>
@@ -453,12 +515,24 @@
     <t>Sistemin kullanılabilirlik hedefleri belirlenmiş mi? Uptime orani, ortalama arisa suresi, ortalama onarim suresi, planli bakim suresi, kesinti tespit suresi, otomatik kurtarma kabiliyeti, yedeklilik, yuk dengeleme, sistem izleme ve alarm</t>
   </si>
   <si>
+    <t>SRS'teki Software System Attributes başlığı altında bulunan tabloda availability metriği tanımlanmıştır.(ör. uptime ≥ 99%, iş akışı retry/queue yapısı) mevcut. Aynı şekilde STP dosyasında bulunan Pass/Fail Criteria başlığında da testlerin nasıl bir sonuç karşısında pass veya fail durumlarının görüleceği tanımlanmıştır.</t>
+  </si>
+  <si>
     <t>3.5.3 Security</t>
   </si>
   <si>
     <t>Güvenlik gereksinimleri açık ve yeterli düzeyde tanımlanmış mı? yetkilendirme, kimlik dogrulama, veri butunlugu, gizlilik, izlenebilirlik, erisim kontrolu, savunma derinligi, saldiri tespiti ve onleme, guvenlik acigi yonetimi, sifreleme</t>
   </si>
   <si>
+    <t>IEEE_SDD v1.1.docx
+Sayfa 9, Interface Descriptions başlığı
+IEEE_SAD v1.0
+Sayfa 7, Physical View başlığı</t>
+  </si>
+  <si>
+    <t>SDD'deki Interface Descriptions başlığı altında MFA prensibi açıklanmış olup sisteme entegre edilecektir. Aynı şekilde SAD dokümanının Physical View başlığı altında bazı güvenlik kısıtları(least privilege, https only, vs.) belirtilmiştir.</t>
+  </si>
+  <si>
     <t>ISO/IEC 27001</t>
   </si>
   <si>
@@ -468,6 +542,15 @@
     <t>Bakım yapılabilirlik gereksinimleri göz önüne alınmış mı? Anasilabilirlik, modulerlik, test edilebilirlik, degistirilebilirlik, uyarlanabilirlik, yinelenen kodlarin azligi, kod standartlarina uygunluk, versiyon kontrolu ve takip, bagimliliklarin yonetimi</t>
   </si>
   <si>
+    <t>IEEE_SAD v1.0
+Sayfa 8-9, Development View başlığı
+IEEE_SRS v2.0
+Sayfa 7-8, Software System Attributes başlığı</t>
+  </si>
+  <si>
+    <t>SDD dokümanında Development View başlığında proje yapısı gösterilmiş, modüleritesi tanımlanmıştır. SRS'teki Software System Atttributes başlığındaki tabloda ise maintainability ile ilgili ifadeler ve hedefler (coupling ratio ≤ 0.25) bulunmaktadır.</t>
+  </si>
+  <si>
     <t>ISO/IEC 14764</t>
   </si>
   <si>
@@ -477,6 +560,9 @@
     <t>Sistemin farklı platformlara taşınabilirliği değerlendirilmiş mi? Platformlar arasi uyum, tasinabilir kod yapisi, kurulum kolayligi, veri uyumlulugu, bagimliliklarin yonetimi, cokli tarayici destegi, mobil uyumluluk, uluslararasilastirma ve yerellestirme, tasinabilir test ortami</t>
   </si>
   <si>
+    <t>SDD dokümanında Deployment Architecture başlığında deployment şekli, kullanılacak araçlar gösterilmiştir. Bu container yapısı ile başka sistemlerde de sıkınıtız çalışması beklenmektedir, bu şekilde portable oluşu sağlanabilir.</t>
+  </si>
+  <si>
     <t>ISO/IEC/IEEE 29119</t>
   </si>
   <si>
@@ -486,12 +572,24 @@
     <t>Ek gereksinimler açıkça listelenmiş mi?</t>
   </si>
   <si>
+    <t>Diğer gereksinimleri içeren bir doküman bulunmamaktadır.</t>
+  </si>
+  <si>
     <t>4.2 Data Collection (If Applicable)</t>
   </si>
   <si>
     <t>Veri toplama yöntemleri ve araçları açıklanmış mı?</t>
   </si>
   <si>
+    <t>IEEE_PMP_v3.0
+Sayfa 6-7, References başlığı
+IEEE_SRS v2.0
+Sayfa 4, Product Perspective ve Product Functions başlıkları</t>
+  </si>
+  <si>
+    <t>PMP ve SRS dokümanlarında hangi veri kaynaklarının kullanılacağı (IDS webhook’ları, mailbox connector, NVD/ExploitDB, malware upload, Caldera telemetry, object storage, MySQL) ve iş akışları açıklanmıştır.</t>
+  </si>
+  <si>
     <t>ISO/IEC 11179</t>
   </si>
   <si>
@@ -501,12 +599,30 @@
     <t>Veri setinin sınırlamaları ve varsayımları belirtilmiş mi?</t>
   </si>
   <si>
+    <t xml:space="preserve">IEEE_PMP_v3.0
+Sayfa 3, Ethical and Legal Risks
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMP'de yer alan Ethical and Legal Risks başlığında datasetler ile ilgili varsayımlar ve sınırlamalar yer alıyor. Kullanılacak açık veri setleri (CICIDS2017, NSL‑KDD, Enron) hakkında bir sınırlama bulunmamaktadır.
+</t>
+  </si>
+  <si>
     <t>6.1 Software Quality Assurance Plan (SQAP)</t>
   </si>
   <si>
     <t>Yazılım kalite güvence planı tanımlanmış mı? amac, kapsam, kalite hedefleri, uygulanacak standartlar, sqa aktiviteleri (kod inceleme, test, surec denetimi, hata izleme etc.), sorumluluklar, dogrulama ve gecerleme, hata ve degisiklik yonetimi, test planlari ve kriterleri, raporlama ve kayit tutma</t>
   </si>
   <si>
+    <t>IEEE_PMP_v3.0
+Sayfa 4-6, Quality Assurance başlığı
+IEEE_STP v1.0.docx
+Sayfa 4-5, Test Approach</t>
+  </si>
+  <si>
+    <t>PMP’de Quality Assurance, STP’de Test Approach başlıkları altında mevcuttur. Kalite etkinliklerinin takibi ve izlenmesi, riskleri, doğrulama süreçleri, hata/değişiklik yöntemleri, açık kalite hedefleri, raporlama formatları yer almaktadır.</t>
+  </si>
+  <si>
     <t>ISO/IEC 12207</t>
   </si>
   <si>
@@ -516,6 +632,14 @@
     <t>Doğrulama ve geçerleme süreçleri açıklanmış mı? Testamaci,basari kriterleri, kullanilan yontemler, test ortami ve kosullari, sonuclarin deerlendirilmesi, iyilestirme onerileri, test katilimcilari, test numarasi ve gereksinim numarasi eslestirme matrisi</t>
   </si>
   <si>
+    <t xml:space="preserve">IEEE_STP v1.0.docx
+Sayfa 3-6, Features to be Tested / Not Tested, Test Approach, Pass/Fail Criteria, Test Deliverables başlıkları
+</t>
+  </si>
+  <si>
+    <t>STP dokümanında V&amp;V ile ilgili parçalar (test amaçları, bazı kabul kriterleri, test seviyeleri, pass/fail kriterleri, traceability başlangıcı) bulunmaktadır. Aynı şekilde Kontrol Listesi 3.2 Functional Requirements bölmesinde yer alan gereksinim eşleme tablosu ile test ve doğrulama süreçleri takip edilebilmektedir.</t>
+  </si>
+  <si>
     <t>IEEE 1012</t>
   </si>
   <si>
@@ -525,6 +649,12 @@
     <t>Yapılandırma yönetimi ve değişiklik takibi nasıl yapılacak belirlenmiş mi?</t>
   </si>
   <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Bulunmamaktadır.</t>
+  </si>
+  <si>
     <t>IEEE 828</t>
   </si>
   <si>
@@ -534,12 +664,25 @@
     <t>Riskler ve hatalar nasıl yönetilecek tanımlanmış mı?</t>
   </si>
   <si>
+    <t xml:space="preserve">IEEE_PMP_v3.0
+Sayfa 3, Risk Management başlığı
+IEEE_STP v1.0.docx
+Sayfa 7, Risks and Contingencies başlığı
+</t>
+  </si>
+  <si>
+    <t>PMP'deki Risk Management ve STP'deki Risks and Contingencies başlıklarında risk ve hata yönetimine dair maddeler(risk listesi, mitigasyon stratejileri, test/triage süreçleri), alınacak aksiyonlar bulunmaktadır.</t>
+  </si>
+  <si>
     <t>6.5 Product Evaluation and Acceptance</t>
   </si>
   <si>
     <t>Ürün kabul kriterleri net ve olculebilir şekilde belirtilmiş mi?</t>
   </si>
   <si>
+    <t>SRS dokümanında yer alan Software System Attributes başlığının altında kabul kriterleri bulunmaktadır, aynı zamanda STP dokümanında bulunan Pass/Fail Criteria ile de testlerin geçilip geçilemediği analiz edilerek eğer SRS'teki koşullarla birlikte uyuşmakta ise kabul sınıfına alınabilir.</t>
+  </si>
+  <si>
     <t>7.3 Risk Analysis and Mitigation Strategies</t>
   </si>
   <si>
@@ -552,10 +695,20 @@
     <t>Hedef kullanıcı kitlesi tanımlanmış mı?</t>
   </si>
   <si>
+    <t>Hedef kullanıcı kitlesi SRS dokümanındaki User Characteristics başlığı altında anlatılmıştır.</t>
+  </si>
+  <si>
     <t>8.2 User Stories</t>
   </si>
   <si>
     <t>Kullanıcı hikayeleri açık ve sistemle uyumlu şekilde tanımlanmış mı? Gereksinim numarasi ve kullanici hikayesi numarasi eslestirme matrisi</t>
+  </si>
+  <si>
+    <t>Üst Seviye Gereksinimlere Bağlı 10 Detaylı Gereksinim(MUDEK_KANIT_15_11_2025)
+Dosyanın tamamı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yan hücrede üst seviye gereksinimlerin bulunduğu doküman bulunmaktadır. Bu dosya en temel use case senaryolarını içererek beraberinde gereksinimleri numaraları ile eşleyerek eşlenebilirliğini sağlamaktadır. </t>
   </si>
   <si>
     <t>9.1 Societal Benefits</t>
@@ -586,6 +739,13 @@
       </rPr>
       <t xml:space="preserve"> etc.</t>
     </r>
+  </si>
+  <si>
+    <t>IEEE_PMP_v3.0
+Sayfa 4-6, Quality Constraints and Risk Register</t>
+  </si>
+  <si>
+    <t>PMP dokümanındaki Quality Constraints and Risk Register başlığında sosyal ve environmental açıdan bahsedilmiştir. Büyük çaplı AI modellerinin eğitilmesinin, optimizasyona olan etkisi, model kalitesine olan etkisi ile environmental açıya değinilirken kullanıcı profiline bağlı olarak kullanılabilite ve data'ların okunabilitesi, yönetilebilmesi açısından sosyal alana da değinilmiştir.</t>
   </si>
   <si>
     <t>9.2 Economic Constraints</t>
@@ -652,6 +812,9 @@
     </r>
   </si>
   <si>
+    <t>PMP dokümanındaki Quality Constraints and Risk Register başlığında ekonomik açıdan bahsedilmiştir. Bu proje üniversite bazlı bir bitirme projesi olması gerekçesi ile yüksek bir bütçe hesaplaması yapılmamış olup gerekli durumlardaki harcamalarda da ekip bütçesi göz önünde bulundurularak ihtiyaçlar(domain, host ücretleri, vs.) değerlendirilecektir.</t>
+  </si>
+  <si>
     <t>9.3 Legal and Ethical Compliance</t>
   </si>
   <si>
@@ -672,6 +835,15 @@
       </rPr>
       <t xml:space="preserve"> kurallara uygunluk sağlanmış mı? Ilgili yasal kurallara , standartlara ve etik ilkelere referans verilmis mi</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">IEEE_PMP_v3.0
+Sayfa 4-6, Quality Constraints and Risk Register
+Sayfa 6, References başlığı
+</t>
+  </si>
+  <si>
+    <t>PMP dokümanındaki Quality Constraints and Risk Register ve References başlıklarında legal ve etik açıdan yaklaşarak kurallara uygunluk sağlanılacağı, yasal sınırlar içerisinde geliştirmelerin yapılacağı belirtilmiştir.</t>
   </si>
 </sst>
 </file>
@@ -744,7 +916,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -781,6 +953,9 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -793,7 +968,36 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="16211550" cy="2305050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Resim"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1157,7 +1361,7 @@
         <v>36</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>13</v>
@@ -1165,16 +1369,16 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>13</v>
@@ -1182,16 +1386,16 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>13</v>
@@ -1199,16 +1403,16 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>13</v>
@@ -1216,1141 +1420,1241 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="6"/>
+        <v>51</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>53</v>
+      </c>
       <c r="E14" s="10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="E15" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="E16" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E17" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" ht="192.0" customHeight="1">
       <c r="A18" s="12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="7"/>
+        <v>68</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>69</v>
+      </c>
       <c r="D18" s="6"/>
       <c r="E18" s="10" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="12" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>74</v>
+      </c>
       <c r="E19" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="12" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="E20" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="12" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>82</v>
+      </c>
       <c r="E21" s="10" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="12" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="6"/>
+        <v>85</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>86</v>
+      </c>
       <c r="E22" s="10" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="12" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="6"/>
+        <v>88</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="E23" s="10" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="12" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="6"/>
+        <v>93</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>95</v>
+      </c>
       <c r="E24" s="10" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="12" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="6"/>
+        <v>98</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>99</v>
+      </c>
       <c r="E25" s="10" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="12" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="C26" s="7"/>
-      <c r="D26" s="6"/>
+      <c r="D26" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="E26" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="12" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="6"/>
+        <v>105</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>107</v>
+      </c>
       <c r="E27" s="10" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="12" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>112</v>
+      </c>
       <c r="E28" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="12" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="6"/>
+        <v>114</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>116</v>
+      </c>
       <c r="E29" s="10" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="12" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="6"/>
+        <v>119</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>121</v>
+      </c>
       <c r="E30" s="10" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="12" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="6"/>
+        <v>124</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>126</v>
+      </c>
       <c r="E31" s="10" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="6"/>
+        <v>129</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>131</v>
+      </c>
       <c r="E32" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="12" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="6"/>
+        <v>133</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>134</v>
+      </c>
       <c r="E33" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="12" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="6"/>
+        <v>136</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>131</v>
+      </c>
       <c r="E34" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="12" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="6"/>
+        <v>138</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>139</v>
+      </c>
       <c r="E35" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="12" t="s">
-        <v>103</v>
+        <v>140</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="6"/>
+        <v>141</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>143</v>
+      </c>
       <c r="E36" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="12" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="6"/>
+        <v>145</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>147</v>
+      </c>
       <c r="E37" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="12" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="6"/>
+        <v>149</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>150</v>
+      </c>
       <c r="E38" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="12" t="s">
-        <v>109</v>
+        <v>151</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="6"/>
+        <v>152</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>154</v>
+      </c>
       <c r="E39" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="15"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="B68" s="14"/>
-      <c r="C68" s="14"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="15"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="B69" s="14"/>
-      <c r="C69" s="14"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
+      <c r="B71" s="15"/>
+      <c r="C71" s="15"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
+      <c r="B72" s="15"/>
+      <c r="C72" s="15"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="15"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="15"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="15"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
+      <c r="B76" s="15"/>
+      <c r="C76" s="15"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="B77" s="14"/>
-      <c r="C77" s="14"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="15"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="B78" s="14"/>
-      <c r="C78" s="14"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="15"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="B80" s="14"/>
-      <c r="C80" s="14"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="15"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="B81" s="14"/>
-      <c r="C81" s="14"/>
+      <c r="B81" s="15"/>
+      <c r="C81" s="15"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="B82" s="14"/>
-      <c r="C82" s="14"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="15"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="B83" s="14"/>
-      <c r="C83" s="14"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="15"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="B84" s="14"/>
-      <c r="C84" s="14"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="15"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="B85" s="14"/>
-      <c r="C85" s="14"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="15"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="B86" s="14"/>
-      <c r="C86" s="14"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="15"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="B87" s="14"/>
-      <c r="C87" s="14"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="15"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="B88" s="14"/>
-      <c r="C88" s="14"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="15"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="B89" s="14"/>
-      <c r="C89" s="14"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="15"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="B90" s="14"/>
-      <c r="C90" s="14"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="15"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="B91" s="14"/>
-      <c r="C91" s="14"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="15"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="B92" s="14"/>
-      <c r="C92" s="14"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="15"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="B93" s="14"/>
-      <c r="C93" s="14"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="15"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="B94" s="14"/>
-      <c r="C94" s="14"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="15"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="B95" s="14"/>
-      <c r="C95" s="14"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="15"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="B96" s="14"/>
-      <c r="C96" s="14"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="15"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="B97" s="14"/>
-      <c r="C97" s="14"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="15"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="B98" s="14"/>
-      <c r="C98" s="14"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="15"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="B99" s="14"/>
-      <c r="C99" s="14"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="15"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="B100" s="14"/>
-      <c r="C100" s="14"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="15"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="B101" s="14"/>
-      <c r="C101" s="14"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="B102" s="14"/>
-      <c r="C102" s="14"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="B103" s="14"/>
-      <c r="C103" s="14"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="15"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="B104" s="14"/>
-      <c r="C104" s="14"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="15"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="B105" s="14"/>
-      <c r="C105" s="14"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="15"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="B106" s="14"/>
-      <c r="C106" s="14"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="15"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="B107" s="14"/>
-      <c r="C107" s="14"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="15"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="B108" s="14"/>
-      <c r="C108" s="14"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="15"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="B109" s="14"/>
-      <c r="C109" s="14"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="15"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="B110" s="14"/>
-      <c r="C110" s="14"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="15"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="B111" s="14"/>
-      <c r="C111" s="14"/>
+      <c r="B111" s="15"/>
+      <c r="C111" s="15"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="B112" s="14"/>
-      <c r="C112" s="14"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="15"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="B113" s="14"/>
-      <c r="C113" s="14"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="15"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="B114" s="14"/>
-      <c r="C114" s="14"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="15"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="B115" s="14"/>
-      <c r="C115" s="14"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="B116" s="14"/>
-      <c r="C116" s="14"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="15"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="B117" s="14"/>
-      <c r="C117" s="14"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="15"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="B118" s="14"/>
-      <c r="C118" s="14"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="15"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="B119" s="14"/>
-      <c r="C119" s="14"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="15"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="B120" s="14"/>
-      <c r="C120" s="14"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="15"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="B121" s="14"/>
-      <c r="C121" s="14"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
-      <c r="B122" s="14"/>
-      <c r="C122" s="14"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
-      <c r="B123" s="14"/>
-      <c r="C123" s="14"/>
+      <c r="B123" s="15"/>
+      <c r="C123" s="15"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
-      <c r="B124" s="14"/>
-      <c r="C124" s="14"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="15"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
-      <c r="B125" s="14"/>
-      <c r="C125" s="14"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="15"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
-      <c r="B126" s="14"/>
-      <c r="C126" s="14"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
-      <c r="B127" s="14"/>
-      <c r="C127" s="14"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="15"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
-      <c r="B128" s="14"/>
-      <c r="C128" s="14"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
-      <c r="B129" s="14"/>
-      <c r="C129" s="14"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="15"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
-      <c r="B130" s="14"/>
-      <c r="C130" s="14"/>
+      <c r="B130" s="15"/>
+      <c r="C130" s="15"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
-      <c r="B131" s="14"/>
-      <c r="C131" s="14"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="15"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
-      <c r="B132" s="14"/>
-      <c r="C132" s="14"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
-      <c r="B133" s="14"/>
-      <c r="C133" s="14"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="15"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
-      <c r="B134" s="14"/>
-      <c r="C134" s="14"/>
+      <c r="B134" s="15"/>
+      <c r="C134" s="15"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
-      <c r="B135" s="14"/>
-      <c r="C135" s="14"/>
+      <c r="B135" s="15"/>
+      <c r="C135" s="15"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
-      <c r="B136" s="14"/>
-      <c r="C136" s="14"/>
+      <c r="B136" s="15"/>
+      <c r="C136" s="15"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
-      <c r="B137" s="14"/>
-      <c r="C137" s="14"/>
+      <c r="B137" s="15"/>
+      <c r="C137" s="15"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
-      <c r="B138" s="14"/>
-      <c r="C138" s="14"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="15"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="B139" s="14"/>
-      <c r="C139" s="14"/>
+      <c r="B139" s="15"/>
+      <c r="C139" s="15"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="B140" s="14"/>
-      <c r="C140" s="14"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="15"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="B141" s="14"/>
-      <c r="C141" s="14"/>
+      <c r="B141" s="15"/>
+      <c r="C141" s="15"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="B142" s="14"/>
-      <c r="C142" s="14"/>
+      <c r="B142" s="15"/>
+      <c r="C142" s="15"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="B143" s="14"/>
-      <c r="C143" s="14"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="15"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="B144" s="14"/>
-      <c r="C144" s="14"/>
+      <c r="B144" s="15"/>
+      <c r="C144" s="15"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="B145" s="14"/>
-      <c r="C145" s="14"/>
+      <c r="B145" s="15"/>
+      <c r="C145" s="15"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="B146" s="14"/>
-      <c r="C146" s="14"/>
+      <c r="B146" s="15"/>
+      <c r="C146" s="15"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="B147" s="14"/>
-      <c r="C147" s="14"/>
+      <c r="B147" s="15"/>
+      <c r="C147" s="15"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="B148" s="14"/>
-      <c r="C148" s="14"/>
+      <c r="B148" s="15"/>
+      <c r="C148" s="15"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="B149" s="14"/>
-      <c r="C149" s="14"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="B150" s="14"/>
-      <c r="C150" s="14"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="15"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="B151" s="14"/>
-      <c r="C151" s="14"/>
+      <c r="B151" s="15"/>
+      <c r="C151" s="15"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="B152" s="14"/>
-      <c r="C152" s="14"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="15"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="B153" s="14"/>
-      <c r="C153" s="14"/>
+      <c r="B153" s="15"/>
+      <c r="C153" s="15"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="B154" s="14"/>
-      <c r="C154" s="14"/>
+      <c r="B154" s="15"/>
+      <c r="C154" s="15"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="B155" s="14"/>
-      <c r="C155" s="14"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="15"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="B156" s="14"/>
-      <c r="C156" s="14"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="15"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="B157" s="14"/>
-      <c r="C157" s="14"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="15"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="B158" s="14"/>
-      <c r="C158" s="14"/>
+      <c r="B158" s="15"/>
+      <c r="C158" s="15"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="B159" s="14"/>
-      <c r="C159" s="14"/>
+      <c r="B159" s="15"/>
+      <c r="C159" s="15"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="B160" s="14"/>
-      <c r="C160" s="14"/>
+      <c r="B160" s="15"/>
+      <c r="C160" s="15"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="B161" s="14"/>
-      <c r="C161" s="14"/>
+      <c r="B161" s="15"/>
+      <c r="C161" s="15"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="B162" s="14"/>
-      <c r="C162" s="14"/>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="B163" s="14"/>
-      <c r="C163" s="14"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="15"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="B164" s="14"/>
-      <c r="C164" s="14"/>
+      <c r="B164" s="15"/>
+      <c r="C164" s="15"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="B165" s="14"/>
-      <c r="C165" s="14"/>
+      <c r="B165" s="15"/>
+      <c r="C165" s="15"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="B166" s="14"/>
-      <c r="C166" s="14"/>
+      <c r="B166" s="15"/>
+      <c r="C166" s="15"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="B167" s="14"/>
-      <c r="C167" s="14"/>
+      <c r="B167" s="15"/>
+      <c r="C167" s="15"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="B168" s="14"/>
-      <c r="C168" s="14"/>
+      <c r="B168" s="15"/>
+      <c r="C168" s="15"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="B169" s="14"/>
-      <c r="C169" s="14"/>
+      <c r="B169" s="15"/>
+      <c r="C169" s="15"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="B170" s="14"/>
-      <c r="C170" s="14"/>
+      <c r="B170" s="15"/>
+      <c r="C170" s="15"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="B171" s="14"/>
-      <c r="C171" s="14"/>
+      <c r="B171" s="15"/>
+      <c r="C171" s="15"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="B172" s="14"/>
-      <c r="C172" s="14"/>
+      <c r="B172" s="15"/>
+      <c r="C172" s="15"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="B173" s="14"/>
-      <c r="C173" s="14"/>
+      <c r="B173" s="15"/>
+      <c r="C173" s="15"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="B174" s="14"/>
-      <c r="C174" s="14"/>
+      <c r="B174" s="15"/>
+      <c r="C174" s="15"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="B175" s="14"/>
-      <c r="C175" s="14"/>
+      <c r="B175" s="15"/>
+      <c r="C175" s="15"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="B176" s="14"/>
-      <c r="C176" s="14"/>
+      <c r="B176" s="15"/>
+      <c r="C176" s="15"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="B177" s="14"/>
-      <c r="C177" s="14"/>
+      <c r="B177" s="15"/>
+      <c r="C177" s="15"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="B178" s="14"/>
-      <c r="C178" s="14"/>
+      <c r="B178" s="15"/>
+      <c r="C178" s="15"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="B179" s="14"/>
-      <c r="C179" s="14"/>
+      <c r="B179" s="15"/>
+      <c r="C179" s="15"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
-      <c r="B180" s="14"/>
-      <c r="C180" s="14"/>
+      <c r="B180" s="15"/>
+      <c r="C180" s="15"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
-      <c r="B181" s="14"/>
-      <c r="C181" s="14"/>
+      <c r="B181" s="15"/>
+      <c r="C181" s="15"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
-      <c r="B182" s="14"/>
-      <c r="C182" s="14"/>
+      <c r="B182" s="15"/>
+      <c r="C182" s="15"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
-      <c r="B183" s="14"/>
-      <c r="C183" s="14"/>
+      <c r="B183" s="15"/>
+      <c r="C183" s="15"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
-      <c r="B184" s="14"/>
-      <c r="C184" s="14"/>
+      <c r="B184" s="15"/>
+      <c r="C184" s="15"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
-      <c r="B185" s="14"/>
-      <c r="C185" s="14"/>
+      <c r="B185" s="15"/>
+      <c r="C185" s="15"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
-      <c r="B186" s="14"/>
-      <c r="C186" s="14"/>
+      <c r="B186" s="15"/>
+      <c r="C186" s="15"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
-      <c r="B187" s="14"/>
-      <c r="C187" s="14"/>
+      <c r="B187" s="15"/>
+      <c r="C187" s="15"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="B188" s="14"/>
-      <c r="C188" s="14"/>
+      <c r="B188" s="15"/>
+      <c r="C188" s="15"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
-      <c r="B189" s="14"/>
-      <c r="C189" s="14"/>
+      <c r="B189" s="15"/>
+      <c r="C189" s="15"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="B190" s="14"/>
-      <c r="C190" s="14"/>
+      <c r="B190" s="15"/>
+      <c r="C190" s="15"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="B191" s="14"/>
-      <c r="C191" s="14"/>
+      <c r="B191" s="15"/>
+      <c r="C191" s="15"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="B192" s="14"/>
-      <c r="C192" s="14"/>
+      <c r="B192" s="15"/>
+      <c r="C192" s="15"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="B193" s="14"/>
-      <c r="C193" s="14"/>
+      <c r="B193" s="15"/>
+      <c r="C193" s="15"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="B194" s="14"/>
-      <c r="C194" s="14"/>
+      <c r="B194" s="15"/>
+      <c r="C194" s="15"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="B195" s="14"/>
-      <c r="C195" s="14"/>
+      <c r="B195" s="15"/>
+      <c r="C195" s="15"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="B196" s="14"/>
-      <c r="C196" s="14"/>
+      <c r="B196" s="15"/>
+      <c r="C196" s="15"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="B197" s="14"/>
-      <c r="C197" s="14"/>
+      <c r="B197" s="15"/>
+      <c r="C197" s="15"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="B198" s="14"/>
-      <c r="C198" s="14"/>
+      <c r="B198" s="15"/>
+      <c r="C198" s="15"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="B199" s="14"/>
-      <c r="C199" s="14"/>
+      <c r="B199" s="15"/>
+      <c r="C199" s="15"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="B200" s="14"/>
-      <c r="C200" s="14"/>
+      <c r="B200" s="15"/>
+      <c r="C200" s="15"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="B201" s="14"/>
-      <c r="C201" s="14"/>
+      <c r="B201" s="15"/>
+      <c r="C201" s="15"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="B202" s="14"/>
-      <c r="C202" s="14"/>
+      <c r="B202" s="15"/>
+      <c r="C202" s="15"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="B203" s="14"/>
-      <c r="C203" s="14"/>
+      <c r="B203" s="15"/>
+      <c r="C203" s="15"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="B204" s="14"/>
-      <c r="C204" s="14"/>
+      <c r="B204" s="15"/>
+      <c r="C204" s="15"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
-      <c r="B205" s="14"/>
-      <c r="C205" s="14"/>
+      <c r="B205" s="15"/>
+      <c r="C205" s="15"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="B206" s="14"/>
-      <c r="C206" s="14"/>
+      <c r="B206" s="15"/>
+      <c r="C206" s="15"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
-      <c r="B207" s="14"/>
-      <c r="C207" s="14"/>
+      <c r="B207" s="15"/>
+      <c r="C207" s="15"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="B208" s="14"/>
-      <c r="C208" s="14"/>
+      <c r="B208" s="15"/>
+      <c r="C208" s="15"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="B209" s="14"/>
-      <c r="C209" s="14"/>
+      <c r="B209" s="15"/>
+      <c r="C209" s="15"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
-      <c r="B210" s="14"/>
-      <c r="C210" s="14"/>
+      <c r="B210" s="15"/>
+      <c r="C210" s="15"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="B211" s="14"/>
-      <c r="C211" s="14"/>
+      <c r="B211" s="15"/>
+      <c r="C211" s="15"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="B212" s="14"/>
-      <c r="C212" s="14"/>
+      <c r="B212" s="15"/>
+      <c r="C212" s="15"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="B213" s="14"/>
-      <c r="C213" s="14"/>
+      <c r="B213" s="15"/>
+      <c r="C213" s="15"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="B214" s="14"/>
-      <c r="C214" s="14"/>
+      <c r="B214" s="15"/>
+      <c r="C214" s="15"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="B215" s="14"/>
-      <c r="C215" s="14"/>
+      <c r="B215" s="15"/>
+      <c r="C215" s="15"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="B216" s="14"/>
-      <c r="C216" s="14"/>
+      <c r="B216" s="15"/>
+      <c r="C216" s="15"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="B217" s="14"/>
-      <c r="C217" s="14"/>
+      <c r="B217" s="15"/>
+      <c r="C217" s="15"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="B218" s="14"/>
-      <c r="C218" s="14"/>
+      <c r="B218" s="15"/>
+      <c r="C218" s="15"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="B219" s="14"/>
-      <c r="C219" s="14"/>
+      <c r="B219" s="15"/>
+      <c r="C219" s="15"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="B220" s="14"/>
-      <c r="C220" s="14"/>
+      <c r="B220" s="15"/>
+      <c r="C220" s="15"/>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="B221" s="14"/>
-      <c r="C221" s="14"/>
+      <c r="B221" s="15"/>
+      <c r="C221" s="15"/>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="B222" s="14"/>
-      <c r="C222" s="14"/>
+      <c r="B222" s="15"/>
+      <c r="C222" s="15"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="B223" s="14"/>
-      <c r="C223" s="14"/>
+      <c r="B223" s="15"/>
+      <c r="C223" s="15"/>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="B224" s="14"/>
-      <c r="C224" s="14"/>
+      <c r="B224" s="15"/>
+      <c r="C224" s="15"/>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="B225" s="14"/>
-      <c r="C225" s="14"/>
+      <c r="B225" s="15"/>
+      <c r="C225" s="15"/>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="B226" s="14"/>
-      <c r="C226" s="14"/>
+      <c r="B226" s="15"/>
+      <c r="C226" s="15"/>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="B227" s="14"/>
-      <c r="C227" s="14"/>
+      <c r="B227" s="15"/>
+      <c r="C227" s="15"/>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="B228" s="14"/>
-      <c r="C228" s="14"/>
+      <c r="B228" s="15"/>
+      <c r="C228" s="15"/>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="B229" s="14"/>
-      <c r="C229" s="14"/>
+      <c r="B229" s="15"/>
+      <c r="C229" s="15"/>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="B230" s="14"/>
-      <c r="C230" s="14"/>
+      <c r="B230" s="15"/>
+      <c r="C230" s="15"/>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="B231" s="14"/>
-      <c r="C231" s="14"/>
+      <c r="B231" s="15"/>
+      <c r="C231" s="15"/>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="B232" s="14"/>
-      <c r="C232" s="14"/>
+      <c r="B232" s="15"/>
+      <c r="C232" s="15"/>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="B233" s="14"/>
-      <c r="C233" s="14"/>
+      <c r="B233" s="15"/>
+      <c r="C233" s="15"/>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="B234" s="14"/>
-      <c r="C234" s="14"/>
+      <c r="B234" s="15"/>
+      <c r="C234" s="15"/>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="B235" s="14"/>
-      <c r="C235" s="14"/>
+      <c r="B235" s="15"/>
+      <c r="C235" s="15"/>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="B236" s="14"/>
-      <c r="C236" s="14"/>
+      <c r="B236" s="15"/>
+      <c r="C236" s="15"/>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="B237" s="14"/>
-      <c r="C237" s="14"/>
+      <c r="B237" s="15"/>
+      <c r="C237" s="15"/>
     </row>
     <row r="238" ht="15.75" customHeight="1">
-      <c r="B238" s="14"/>
-      <c r="C238" s="14"/>
+      <c r="B238" s="15"/>
+      <c r="C238" s="15"/>
     </row>
     <row r="239" ht="15.75" customHeight="1">
-      <c r="B239" s="14"/>
-      <c r="C239" s="14"/>
+      <c r="B239" s="15"/>
+      <c r="C239" s="15"/>
     </row>
     <row r="240" ht="15.75" customHeight="1"/>
     <row r="241" ht="15.75" customHeight="1"/>
@@ -3126,7 +3430,30 @@
     <hyperlink r:id="rId9" ref="C11"/>
     <hyperlink r:id="rId10" ref="C12"/>
     <hyperlink r:id="rId11" ref="C13"/>
+    <hyperlink r:id="rId12" ref="C14"/>
+    <hyperlink r:id="rId13" ref="C15"/>
+    <hyperlink r:id="rId14" ref="C16"/>
+    <hyperlink r:id="rId15" ref="C17"/>
+    <hyperlink r:id="rId16" ref="C19"/>
+    <hyperlink r:id="rId17" ref="C20"/>
+    <hyperlink r:id="rId18" ref="C21"/>
+    <hyperlink r:id="rId19" ref="C22"/>
+    <hyperlink r:id="rId20" ref="C23"/>
+    <hyperlink r:id="rId21" ref="C24"/>
+    <hyperlink r:id="rId22" ref="C25"/>
+    <hyperlink r:id="rId23" ref="C27"/>
+    <hyperlink r:id="rId24" ref="C28"/>
+    <hyperlink r:id="rId25" ref="C29"/>
+    <hyperlink r:id="rId26" ref="C30"/>
+    <hyperlink r:id="rId27" ref="C32"/>
+    <hyperlink r:id="rId28" ref="C33"/>
+    <hyperlink r:id="rId29" ref="C34"/>
+    <hyperlink r:id="rId30" ref="C35"/>
+    <hyperlink r:id="rId31" ref="C36"/>
+    <hyperlink r:id="rId32" ref="C37"/>
+    <hyperlink r:id="rId33" ref="C38"/>
+    <hyperlink r:id="rId34" ref="C39"/>
   </hyperlinks>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>